<commit_message>
Added review index for stricter de-duplication sensitivity analysis
</commit_message>
<xml_diff>
--- a/ReviewIndex_Final.xlsx
+++ b/ReviewIndex_Final.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2178448209088/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_17DC7ED08F79A8D366075C52F37BD272FA45DE2F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8AC927D-20A4-F54B-A8A1-7644FC4A377C}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_17DC7ED08F79A8D366075C52F37BD272FA45DE2F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BA67BA7-CC42-0D48-8350-1CDF90485B74}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="840" windowWidth="50720" windowHeight="27720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="280" yWindow="980" windowWidth="33640" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
     <sheet name="CountryRegions" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Main!$K$1:$K$91</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>

</xml_diff>